<commit_message>
feat(v0.4): implement MASTER-first architecture
</commit_message>
<xml_diff>
--- a/output/RESULT.xlsx
+++ b/output/RESULT.xlsx
@@ -476,7 +476,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>BABY</t>
+          <t>ПАРФЮМИРОВАННЫЙ BABY</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MIDNIGHT</t>
+          <t>ПАРФЮМИРОВАННЫЙ MIDNIGHT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -560,7 +560,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>VELVET</t>
+          <t>ПАРФЮМИРОВАННЫЙ VELVET</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -602,7 +602,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>FLORAL MIST</t>
+          <t>ПАРФЮМИРОВАННЫЙ FLORAL MIST</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SWEET TROPIC</t>
+          <t>ПАРФЮМИРОВАННЫЙ SWEET TROPIC</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -686,7 +686,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DREAM</t>
+          <t>ПАРФЮМИРОВАННЫЙ DREAM</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>BLACK</t>
+          <t>ПАРФЮМИРОВАННЫЙ BLACK</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -770,7 +770,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>SHAFRAN</t>
+          <t>ПАРФЮМИРОВАННЫЙ SHAFRAN</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -778,9 +778,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>SKU-032</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Saffran 1 л</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -802,7 +812,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>() 2 ПИОН</t>
+          <t>ПАРФЮМИРОВАННЫЙ () 2 ПИОН</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -834,7 +844,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>() 2 ГОРНЫЙ БРИЗ</t>
+          <t>ПАРФЮМИРОВАННЫ() 2 ГОРНЫЙ БРИЗ</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -866,7 +876,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>() 2 АРОМАТ ЦВЕТОВ</t>
+          <t>ПАРФЮМИРОВАННЫЙ() 2 АРОМАТ ЦВЕТОВ</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -898,7 +908,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>ВАНИЛЬ () 2</t>
+          <t>ПАРФЮМИРОВАННЫЙ ВАНИЛЬ () 2</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -930,7 +940,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ЛАВАНДА () 2</t>
+          <t>ПАРФЮМИРОВАННЫЙ ЛАВАНДА () 2</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -962,7 +972,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>РОЗА () 2</t>
+          <t>ПАРФЮМИРОВАННЫЙ РОЗА () 2</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -994,7 +1004,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>РОМАШКА PAPATYA 2</t>
+          <t>ПАРФЮМИРОВАННЫЙ РОМАШКА PAPATYA 2</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1002,9 +1012,19 @@
           <t>7 л</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>SKU-040</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Papatya 1,44 л</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1046,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ПОЛНОЧЬ MIDNIGHT 2</t>
+          <t>ПАРФЮМИРОВАННЫЙ ПОЛНОЧЬ MIDNIGHT 2</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1034,9 +1054,19 @@
           <t>7 л</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>SKU-026</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Midnight 1 л</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1088,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>АРОМАТ СТРАСТИ DAHLIA 2</t>
+          <t>ПАРФЮМИРОВАННЫЙ АРОМАТ СТРАСТИ DAHLIA 2</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1090,7 +1120,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>ТАИНСТВЕННЫЙ ЛОТОС LOTOS</t>
+          <t>ПАРФЮМИРОВАННЫЙ ТАИНСТВЕННЫЙ ЛОТОС LOTOS</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1117,7 +1147,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ЦВЕТОЧНЫЙ ТУМАН FLORIAL 2 7</t>
+          <t>ПАРФЮМИРОВАННЫЙ ЦВЕТОЧНЫЙ ТУМАН FLORIAL 2 7</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1144,7 +1174,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>МАНГО MANGO 2</t>
+          <t>ПАРФЮМИРОВАННЫЙ МАНГО MANGO 2</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1176,7 +1206,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>ДЛЯ ТЕМНОГО БЕЛЬЯ 2</t>
+          <t>ПАРФЮМИРОВАННЫЙ ДЛЯ ТЕМНОГО БЕЛЬЯ 2</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1238,9 +1268,19 @@
           <t>400 мл</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>SKU-009</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Шампунь men GILAR Keratin Extracts 400 мл</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -1314,9 +1354,19 @@
           <t>400 мл</t>
         </is>
       </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>SKU-013</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Шампунь sport GILAR Blue 400 мл</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -1346,9 +1396,19 @@
           <t>400 мл</t>
         </is>
       </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>SKU-012</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Шампунь sport GILAR Black 400 мл</t>
+        </is>
+      </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -1607,9 +1667,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>SKU-262</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Pomegranate 1 л</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -1634,9 +1704,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>SKU-262</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Pomegranate 1 л</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -1661,9 +1741,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>SKU-028</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Floral Mist 1 л</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -1688,9 +1778,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>SKU-026</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Midnight 1 л</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -1715,9 +1815,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>SKU-029</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Sweet Tropic 1 л</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -1742,9 +1852,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>SKU-029</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Sweet Tropic 1 л</t>
+        </is>
+      </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -1769,9 +1889,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>SKU-027</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Velvet 1 л</t>
+        </is>
+      </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -1796,9 +1926,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>SKU-262</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Pomegranate 1 л</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -1985,9 +2125,19 @@
           <t>2 л</t>
         </is>
       </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>SKU-270</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Orange 2 л</t>
+        </is>
+      </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2012,9 +2162,19 @@
           <t>2 л</t>
         </is>
       </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>SKU-271</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Lemon 2 л</t>
+        </is>
+      </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2039,9 +2199,19 @@
           <t>2 л</t>
         </is>
       </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>SKU-272</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Wild Berries 2 л</t>
+        </is>
+      </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2066,9 +2236,19 @@
           <t>2 л</t>
         </is>
       </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>SKU-273</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Apple 2 л</t>
+        </is>
+      </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2093,9 +2273,19 @@
           <t>2 л</t>
         </is>
       </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>SKU-274</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Ginger 2 л</t>
+        </is>
+      </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2120,9 +2310,19 @@
           <t>2 л</t>
         </is>
       </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>SKU-275</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Passion Fruit 2 л</t>
+        </is>
+      </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2147,9 +2347,19 @@
           <t>2 л</t>
         </is>
       </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>SKU-276</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Pomegranate 2 л</t>
+        </is>
+      </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2174,9 +2384,19 @@
           <t>2 л</t>
         </is>
       </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>SKU-277</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Strawberry 2 л</t>
+        </is>
+      </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2201,9 +2421,19 @@
           <t>2 л</t>
         </is>
       </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>SKU-278</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Mango 2 л</t>
+        </is>
+      </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2390,9 +2620,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>SKU-073</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Love Is 5 л</t>
+        </is>
+      </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2417,9 +2657,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>SKU-073</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Love Is 5 л</t>
+        </is>
+      </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2636,9 +2886,19 @@
           <t>500 мл</t>
         </is>
       </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>SKU-114</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Жидкое мыло SVO Passion Fruit 500 мл</t>
+        </is>
+      </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2663,9 +2923,19 @@
           <t>500 мл</t>
         </is>
       </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>SKU-115</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Жидкое мыло SVO Chocolate 500 мл</t>
+        </is>
+      </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2690,9 +2960,19 @@
           <t>500 мл</t>
         </is>
       </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>SKU-116</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Жидкое мыло SVO Mango 500 мл</t>
+        </is>
+      </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2717,9 +2997,19 @@
           <t>500 мл</t>
         </is>
       </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>SKU-117</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Жидкое мыло SVO Wild Berries 500 мл</t>
+        </is>
+      </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2744,9 +3034,19 @@
           <t>500 мл</t>
         </is>
       </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>SKU-118</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Крем-мыло GILAR Coconut 500 мл</t>
+        </is>
+      </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2771,9 +3071,19 @@
           <t>500 мл</t>
         </is>
       </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>SKU-119</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Крем-мыло GILAR Oatmeal 500 мл</t>
+        </is>
+      </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2798,9 +3108,19 @@
           <t>500 мл</t>
         </is>
       </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>SKU-120</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Крем-мыло GILAR Oriental 500 мл</t>
+        </is>
+      </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2825,9 +3145,19 @@
           <t>500 мл</t>
         </is>
       </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>SKU-121</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Крем-мыло GILAR Pine Forest 500 мл</t>
+        </is>
+      </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2852,9 +3182,19 @@
           <t>500 мл</t>
         </is>
       </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>SKU-122</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Крем-мыло GILAR Cherry 500 мл</t>
+        </is>
+      </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2884,9 +3224,19 @@
           <t>600 мл</t>
         </is>
       </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>SKU-014</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Шампунь GILAR Almond 600 мл</t>
+        </is>
+      </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2916,9 +3266,19 @@
           <t>600 мл</t>
         </is>
       </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>SKU-015</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Шампунь GILAR Aloe Vera 600 мл</t>
+        </is>
+      </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2948,9 +3308,19 @@
           <t>600 мл</t>
         </is>
       </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>SKU-016</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Шампунь GILAR Garlic 600 мл</t>
+        </is>
+      </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -2980,9 +3350,19 @@
           <t>600 мл</t>
         </is>
       </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>SKU-017</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Шампунь GILAR Keratin 600 мл</t>
+        </is>
+      </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -3012,9 +3392,19 @@
           <t>600 мл</t>
         </is>
       </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>SKU-018</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Шампунь GILAR Mint 600 мл</t>
+        </is>
+      </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -3044,9 +3434,19 @@
           <t>600 мл</t>
         </is>
       </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>SKU-019</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Шампунь GILAR Nettle 600 мл</t>
+        </is>
+      </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -4843,9 +5243,19 @@
           <t>BOSSFIX</t>
         </is>
       </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>SKU-082</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>ЖМС BOSSFIX Baby 1 л</t>
+        </is>
+      </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -4860,9 +5270,19 @@
           <t>BOSSFIX</t>
         </is>
       </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>SKU-082</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>ЖМС BOSSFIX Baby 1 л</t>
+        </is>
+      </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -4884,7 +5304,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>MAGINA АРАБСКИЙ ПАРФЮМ 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ MAGINA АРАБСКИЙ ПАРФЮМ 1</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
@@ -4916,7 +5336,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>VELVET 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ VELVET 1</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
@@ -4924,9 +5344,19 @@
           <t>44 л</t>
         </is>
       </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>SKU-027</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Velvet 1 л</t>
+        </is>
+      </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -4948,7 +5378,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>ЛОТОС 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ ЛОТОС 1</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
@@ -4980,7 +5410,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>МАНГО 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ МАНГО 1</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
@@ -5012,7 +5442,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>DREAM 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ DREAM 1</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
@@ -5020,9 +5450,19 @@
           <t>44 л</t>
         </is>
       </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>SKU-030</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Dream 1 л</t>
+        </is>
+      </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5044,7 +5484,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>MIDNIGHT 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ MIDNIGHT 1</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
@@ -5052,9 +5492,19 @@
           <t>44 л</t>
         </is>
       </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>SKU-026</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Midnight 1 л</t>
+        </is>
+      </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5526,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>TUTKULU DOHLIA СТРАСТИ 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ TUTKULU DOHLIA СТРАСТИ 1</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
@@ -5084,9 +5534,19 @@
           <t>44 л</t>
         </is>
       </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>SKU-039</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Tutkulu Dahlia 1,44 л</t>
+        </is>
+      </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5108,7 +5568,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>PAPATYE РОМАШКА 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ PAPATYE РОМАШКА 1</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
@@ -5116,9 +5576,19 @@
           <t>44 л</t>
         </is>
       </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>SKU-040</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Papatya 1,44 л</t>
+        </is>
+      </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5610,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>FLORAL MIST 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ FLORAL MIST 1</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
@@ -5148,9 +5618,19 @@
           <t>44 л</t>
         </is>
       </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>SKU-028</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Floral Mist 1 л</t>
+        </is>
+      </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5172,7 +5652,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>PASSION FRUIT МАРАКУЙЯ 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ PASSION FRUIT МАРАКУЙЯ 1</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
@@ -5180,9 +5660,19 @@
           <t>44 л</t>
         </is>
       </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>SKU-042</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Passion Fruit 1,44 л</t>
+        </is>
+      </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5204,7 +5694,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>ORCHIDE ОРХИДЕЯ 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ ORCHIDE ОРХИДЕЯ 1</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
@@ -5212,9 +5702,19 @@
           <t>44 л</t>
         </is>
       </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>SKU-043</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Orchide 1,44 л</t>
+        </is>
+      </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5236,7 +5736,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>SAFFRAN ШАФРАН 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ SAFFRAN ШАФРАН 1</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
@@ -5244,9 +5744,19 @@
           <t>44 л</t>
         </is>
       </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>SKU-032</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Saffran 1 л</t>
+        </is>
+      </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5268,7 +5778,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>SHAIK ШЕЙХ 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ SHAIK ШЕЙХ 1</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
@@ -5276,9 +5786,19 @@
           <t>44 л</t>
         </is>
       </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>SKU-045</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Shaik 1,44 л</t>
+        </is>
+      </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5820,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>JASMIN ЖАСМИН 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ JASMIN ЖАСМИН 1</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
@@ -5308,9 +5828,19 @@
           <t>44 л</t>
         </is>
       </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>SKU-046</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Jasmin 1,44 л</t>
+        </is>
+      </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5332,12 +5862,22 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>ROMANTIK ROSE РОМАНТИЧНАЯ РОЗА 1 44</t>
+          <t>ПАРФЮМИРОВАННЫЙ ROMANTIK ROSE РОМАНТИЧНАЯ РОЗА 1 44</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>SKU-047</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Romantik Rose 1,44 л</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5359,7 +5899,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>SWEET TROPIC 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ SWEET TROPIC 1</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
@@ -5367,9 +5907,19 @@
           <t>44 л</t>
         </is>
       </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>SKU-029</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Sweet Tropic 1 л</t>
+        </is>
+      </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5391,7 +5941,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>ROSE РОЗА 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ ROSE РОЗА 1</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
@@ -5423,7 +5973,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>BOTANIC СЕНТЯБРЬСКОЕ СОЛНЦЕ 1</t>
+          <t>BOTANIC ПАРФЮМИРОВАННЫЙ СЕНТЯБРЬСКОЕ СОЛНЦЕ 1</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
@@ -5455,7 +6005,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>BOTANIC ДОЖДЛИВЫЙ АПРЕЛЬ 1</t>
+          <t>BOTANIC ПАРФЮМИРОВАННЫЙ ДОЖДЛИВЫЙ АПРЕЛЬ 1</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
@@ -5487,7 +6037,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>BLACKBERRY ЕЖЕВИКА 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ BLACKBERRY ЕЖЕВИКА 1</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
@@ -5495,9 +6045,19 @@
           <t>44 л</t>
         </is>
       </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>SKU-052</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Blackberry 1,44 л</t>
+        </is>
+      </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5519,7 +6079,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>BABY ДЕТСКИЙ 1</t>
+          <t>ПАРФЮМИРОВАННЫЙ BABY ДЕТСКИЙ 1</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
@@ -5586,9 +6146,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>SKU-073</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Love Is 5 л</t>
+        </is>
+      </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5613,9 +6183,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>SKU-072</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Maiden Tower 5 л</t>
+        </is>
+      </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5640,9 +6220,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>SKU-073</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Love Is 5 л</t>
+        </is>
+      </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5667,9 +6257,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>SKU-072</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Maiden Tower 5 л</t>
+        </is>
+      </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5694,9 +6294,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>SKU-073</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Love Is 5 л</t>
+        </is>
+      </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5721,9 +6331,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>SKU-072</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Maiden Tower 5 л</t>
+        </is>
+      </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5748,9 +6368,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>SKU-069</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Frezya 5 л</t>
+        </is>
+      </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5775,9 +6405,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>SKU-073</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Love Is 5 л</t>
+        </is>
+      </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5802,9 +6442,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>SKU-073</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Love Is 5 л</t>
+        </is>
+      </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5829,9 +6479,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>SKU-068</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Ask 5 л</t>
+        </is>
+      </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5856,9 +6516,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>SKU-072</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Maiden Tower 5 л</t>
+        </is>
+      </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5883,9 +6553,19 @@
           <t>3 л</t>
         </is>
       </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>SKU-094</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>ЖМС SVO Midnight 3 л</t>
+        </is>
+      </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5910,9 +6590,19 @@
           <t>3 л</t>
         </is>
       </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>SKU-095</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>ЖМС SVO Dream 3 л</t>
+        </is>
+      </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5937,9 +6627,19 @@
           <t>3 л</t>
         </is>
       </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>SKU-096</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>ЖМС SVO Velvet 3 л</t>
+        </is>
+      </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -5991,9 +6691,19 @@
           <t>3 л</t>
         </is>
       </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>SKU-098</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>ЖМС SVO Black 3 л</t>
+        </is>
+      </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6018,9 +6728,19 @@
           <t>3 л</t>
         </is>
       </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>SKU-099</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>ЖМС SVO Color 3 л</t>
+        </is>
+      </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6045,9 +6765,19 @@
           <t>3 л</t>
         </is>
       </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>SKU-100</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>ЖМС SVO White 3 л</t>
+        </is>
+      </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6158,9 +6888,19 @@
           <t>500 мл</t>
         </is>
       </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>SKU-020</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>Шампунь органический GILAR Argan Oil 500 мл</t>
+        </is>
+      </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6190,9 +6930,19 @@
           <t>500 мл</t>
         </is>
       </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>SKU-021</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>Шампунь органический GILAR Coffee 500 мл</t>
+        </is>
+      </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6222,9 +6972,19 @@
           <t>500 мл</t>
         </is>
       </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>SKU-022</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>Шампунь органический GILAR Ginger 500 мл</t>
+        </is>
+      </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6254,9 +7014,19 @@
           <t>500 мл</t>
         </is>
       </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>SKU-023</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>Шампунь органический GILAR Lavender 500 мл</t>
+        </is>
+      </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6286,9 +7056,19 @@
           <t>500 мл</t>
         </is>
       </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>SKU-024</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>Шампунь органический GILAR Ginseng 500 мл</t>
+        </is>
+      </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6313,9 +7093,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>SKU-261</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Orange 1 л</t>
+        </is>
+      </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6340,9 +7130,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>SKU-262</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Pomegranate 1 л</t>
+        </is>
+      </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6367,9 +7167,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>SKU-263</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Wild Berries 1 л</t>
+        </is>
+      </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6394,9 +7204,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>SKU-264</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Ginger 1 л</t>
+        </is>
+      </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6421,9 +7241,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>SKU-265</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Strawberry 1 л</t>
+        </is>
+      </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6448,9 +7278,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>SKU-266</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Lemon 1 л</t>
+        </is>
+      </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6475,9 +7315,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>SKU-267</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Mango 1 л</t>
+        </is>
+      </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6502,9 +7352,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>SKU-268</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Passion 1 л</t>
+        </is>
+      </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6529,9 +7389,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>SKU-269</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>Посуда моющее ср-во SVO Apple 1 л</t>
+        </is>
+      </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6553,7 +7423,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>ASK ЛЮБОВЬ</t>
+          <t>ПАРФЮМИРОВАННЫЙ ASK ЛЮБОВЬ</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
@@ -6561,9 +7431,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>SKU-068</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Ask 5 л</t>
+        </is>
+      </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6585,7 +7465,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>FREZYA ИРИС</t>
+          <t>ПАРФЮМИРОВАННЫЙ FREZYA ИРИС</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
@@ -6593,9 +7473,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>SKU-069</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Frezya 5 л</t>
+        </is>
+      </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6617,7 +7507,7 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>GUL РОЗА</t>
+          <t>ПАРФЮМИРОВАННЫЙ GUL РОЗА</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
@@ -6625,9 +7515,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>SKU-070</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Gul 5 л</t>
+        </is>
+      </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6649,7 +7549,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>HUZUR УСПОКАИВАЮЩИЙ</t>
+          <t>ПАРФЮМИРОВАННЫЙ HUZUR УСПОКАИВАЮЩИЙ</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
@@ -6657,9 +7557,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>SKU-071</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Huzur 5 л</t>
+        </is>
+      </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6681,7 +7591,7 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>MAIDEN TOWER ОРХИДЕЯ</t>
+          <t>ПАРФЮМИРОВАННЫЙ MAIDEN TOWER ОРХИДЕЯ</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
@@ -6689,9 +7599,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>SKU-072</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Maiden Tower 5 л</t>
+        </is>
+      </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6713,7 +7633,7 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>LOVE IS ЦВЕТОЧНЫЙ</t>
+          <t>ПАРФЮМИРОВАННЫЙ LOVE IS ЦВЕТОЧНЫЙ</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
@@ -6721,9 +7641,19 @@
           <t>5 л</t>
         </is>
       </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>SKU-073</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Love Is 5 л</t>
+        </is>
+      </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -6838,9 +7768,19 @@
           <t>500 мл</t>
         </is>
       </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>SKU-020</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>Шампунь органический GILAR Argan Oil 500 мл</t>
+        </is>
+      </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -7235,9 +8175,19 @@
           <t>7 л</t>
         </is>
       </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>SKU-039</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Tutkulu Dahlia 1,44 л</t>
+        </is>
+      </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -7267,9 +8217,19 @@
           <t>7 л</t>
         </is>
       </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>SKU-059</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Lavender 2,7 л</t>
+        </is>
+      </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -7294,9 +8254,19 @@
           <t>РОМАНТИЧЕСКИЙ АРОМАТ ROMANTIK GUL 3В1</t>
         </is>
       </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>SKU-047</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Romantik Rose 1,44 л</t>
+        </is>
+      </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -7326,9 +8296,19 @@
           <t>7 л</t>
         </is>
       </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>SKU-028</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Floral Mist 1 л</t>
+        </is>
+      </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -7358,9 +8338,19 @@
           <t>7 л</t>
         </is>
       </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>SKU-067</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Black Gel 2,7 л</t>
+        </is>
+      </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -7390,9 +8380,19 @@
           <t>7 л</t>
         </is>
       </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>SKU-026</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Midnight 1 л</t>
+        </is>
+      </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -7407,9 +8407,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>SKU-025</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Baby 1 л</t>
+        </is>
+      </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -7424,9 +8434,19 @@
           <t>1 л</t>
         </is>
       </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>SKU-025</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Baby 1 л</t>
+        </is>
+      </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCH</t>
         </is>
       </c>
     </row>

</xml_diff>